<commit_message>
EPBDS-16529 Cover the types the input array lookup accepts
The index was tested on strings and on a numeric cast only. The tests now
cover a path to the array, a primitive and a boxed array of inputs, dates and
an alias type in the condition column.
</commit_message>
<xml_diff>
--- a/DEV/org.openl.rules.test/test-resources/functionality/EPBDS-16529_DecisionTable_ContainsInInputArrayIndex.xlsx
+++ b/DEV/org.openl.rules.test/test-resources/functionality/EPBDS-16529_DecisionTable_ContainsInInputArrayIndex.xlsx
@@ -471,7 +471,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J77"/>
+  <dimension ref="A1:J143"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="2" max="2"/>
@@ -1742,21 +1742,809 @@
         </is>
       </c>
     </row>
+    <row r="78"/>
+    <row r="79"/>
+    <row r="80">
+      <c r="H80" s="1" t="inlineStr">
+        <is>
+          <t>Test selectByCodeOfCoverage selectByCodeOfCoverageTest</t>
+        </is>
+      </c>
+      <c r="I80" s="2" t="n"/>
+    </row>
+    <row r="81">
+      <c r="B81" s="1" t="inlineStr">
+        <is>
+          <t>Datatype Coverage</t>
+        </is>
+      </c>
+      <c r="C81" s="2" t="n"/>
+      <c r="H81" s="4" t="inlineStr">
+        <is>
+          <t>coverage.codes</t>
+        </is>
+      </c>
+      <c r="I81" s="4" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>String[]</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>codes</t>
+        </is>
+      </c>
+      <c r="H82" s="4" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="I82" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="H83" s="5" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="I83" s="5" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="H84" s="5" t="inlineStr">
+        <is>
+          <t>unknown</t>
+        </is>
+      </c>
+      <c r="I84" s="5" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+    </row>
+    <row r="85">
+      <c r="H85" s="6" t="n"/>
+      <c r="I85" s="5" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+    </row>
+    <row r="86">
+      <c r="B86" s="1" t="inlineStr">
+        <is>
+          <t>Rules String selectByCodeOfCoverage(Coverage coverage)</t>
+        </is>
+      </c>
+      <c r="C86" s="2" t="n"/>
+    </row>
+    <row r="87">
+      <c r="B87" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C87" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="88">
+      <c r="B88" s="4" t="inlineStr">
+        <is>
+          <t>contains(coverage.codes, code)</t>
+        </is>
+      </c>
+      <c r="C88" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="89">
+      <c r="B89" s="4" t="inlineStr">
+        <is>
+          <t>String code</t>
+        </is>
+      </c>
+      <c r="C89" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+      <c r="H89" s="1" t="inlineStr">
+        <is>
+          <t>Test selectById selectByIdTest</t>
+        </is>
+      </c>
+      <c r="I89" s="2" t="n"/>
+    </row>
+    <row r="90">
+      <c r="B90" s="4" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C90" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="H90" s="4" t="inlineStr">
+        <is>
+          <t>ids</t>
+        </is>
+      </c>
+      <c r="I90" s="4" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="91">
+      <c r="B91" s="5" t="inlineStr">
+        <is>
+          <t>foo</t>
+        </is>
+      </c>
+      <c r="C91" s="5" t="inlineStr">
+        <is>
+          <t>Foo</t>
+        </is>
+      </c>
+      <c r="H91" s="4" t="inlineStr">
+        <is>
+          <t>Ids</t>
+        </is>
+      </c>
+      <c r="I91" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="92">
+      <c r="B92" s="5" t="inlineStr">
+        <is>
+          <t>bar</t>
+        </is>
+      </c>
+      <c r="C92" s="5" t="inlineStr">
+        <is>
+          <t>Bar</t>
+        </is>
+      </c>
+      <c r="H92" s="5" t="inlineStr">
+        <is>
+          <t>9,2</t>
+        </is>
+      </c>
+      <c r="I92" s="5" t="inlineStr">
+        <is>
+          <t>Two</t>
+        </is>
+      </c>
+    </row>
+    <row r="93">
+      <c r="B93" s="6" t="n"/>
+      <c r="C93" s="5" t="inlineStr">
+        <is>
+          <t>Any</t>
+        </is>
+      </c>
+      <c r="H93" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I93" s="5" t="inlineStr">
+        <is>
+          <t>One</t>
+        </is>
+      </c>
+    </row>
+    <row r="94">
+      <c r="H94" s="5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I94" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="95"/>
+    <row r="96"/>
+    <row r="97">
+      <c r="B97" s="1" t="inlineStr">
+        <is>
+          <t>Rules String selectById(int[] ids)</t>
+        </is>
+      </c>
+      <c r="C97" s="2" t="n"/>
+    </row>
+    <row r="98">
+      <c r="B98" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C98" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+      <c r="H98" s="1" t="inlineStr">
+        <is>
+          <t>Test selectByBoxedId selectByBoxedIdTest</t>
+        </is>
+      </c>
+      <c r="I98" s="2" t="n"/>
+    </row>
+    <row r="99">
+      <c r="B99" s="4" t="inlineStr">
+        <is>
+          <t>contains(ids, id)</t>
+        </is>
+      </c>
+      <c r="C99" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="H99" s="4" t="inlineStr">
+        <is>
+          <t>ids</t>
+        </is>
+      </c>
+      <c r="I99" s="4" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="100">
+      <c r="B100" s="4" t="inlineStr">
+        <is>
+          <t>Integer id</t>
+        </is>
+      </c>
+      <c r="C100" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+      <c r="H100" s="4" t="inlineStr">
+        <is>
+          <t>Ids</t>
+        </is>
+      </c>
+      <c r="I100" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="B101" s="4" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="C101" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="H101" s="5" t="inlineStr">
+        <is>
+          <t>9,2</t>
+        </is>
+      </c>
+      <c r="I101" s="5" t="inlineStr">
+        <is>
+          <t>Two</t>
+        </is>
+      </c>
+    </row>
+    <row r="102">
+      <c r="B102" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C102" s="5" t="inlineStr">
+        <is>
+          <t>One</t>
+        </is>
+      </c>
+      <c r="H102" s="5" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="I102" s="5" t="inlineStr">
+        <is>
+          <t>One</t>
+        </is>
+      </c>
+    </row>
+    <row r="103">
+      <c r="B103" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C103" s="5" t="inlineStr">
+        <is>
+          <t>Two</t>
+        </is>
+      </c>
+      <c r="H103" s="5" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
+      <c r="I103" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="104">
+      <c r="B104" s="6" t="n"/>
+      <c r="C104" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="105"/>
+    <row r="106"/>
+    <row r="107">
+      <c r="H107" s="1" t="inlineStr">
+        <is>
+          <t>Test selectByDate selectByDateTest</t>
+        </is>
+      </c>
+      <c r="I107" s="2" t="n"/>
+    </row>
+    <row r="108">
+      <c r="B108" s="1" t="inlineStr">
+        <is>
+          <t>Rules String selectByBoxedId(Integer[] ids)</t>
+        </is>
+      </c>
+      <c r="C108" s="2" t="n"/>
+      <c r="H108" s="4" t="inlineStr">
+        <is>
+          <t>dates</t>
+        </is>
+      </c>
+      <c r="I108" s="4" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="B109" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C109" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+      <c r="H109" s="4" t="inlineStr">
+        <is>
+          <t>Dates</t>
+        </is>
+      </c>
+      <c r="I109" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="110">
+      <c r="B110" s="4" t="inlineStr">
+        <is>
+          <t>contains(ids, id)</t>
+        </is>
+      </c>
+      <c r="C110" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="H110" s="5" t="inlineStr">
+        <is>
+          <t>12/12/2021,03/04/2020</t>
+        </is>
+      </c>
+      <c r="I110" s="5" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+    </row>
+    <row r="111">
+      <c r="B111" s="4" t="inlineStr">
+        <is>
+          <t>int id</t>
+        </is>
+      </c>
+      <c r="C111" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+      <c r="H111" s="5" t="inlineStr">
+        <is>
+          <t>01/02/2020</t>
+        </is>
+      </c>
+      <c r="I111" s="5" t="inlineStr">
+        <is>
+          <t>First</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="B112" s="4" t="inlineStr">
+        <is>
+          <t>Id</t>
+        </is>
+      </c>
+      <c r="C112" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+      <c r="H112" s="5" t="inlineStr">
+        <is>
+          <t>12/12/2021</t>
+        </is>
+      </c>
+      <c r="I112" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="B113" s="5" t="n">
+        <v>1</v>
+      </c>
+      <c r="C113" s="5" t="inlineStr">
+        <is>
+          <t>One</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="B114" s="5" t="n">
+        <v>2</v>
+      </c>
+      <c r="C114" s="5" t="inlineStr">
+        <is>
+          <t>Two</t>
+        </is>
+      </c>
+    </row>
+    <row r="115">
+      <c r="B115" s="6" t="n"/>
+      <c r="C115" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="116">
+      <c r="H116" s="1" t="inlineStr">
+        <is>
+          <t>Test selectByCoverageCode selectByCoverageCodeTest</t>
+        </is>
+      </c>
+      <c r="I116" s="2" t="n"/>
+    </row>
+    <row r="117">
+      <c r="H117" s="4" t="inlineStr">
+        <is>
+          <t>codes</t>
+        </is>
+      </c>
+      <c r="I117" s="4" t="inlineStr">
+        <is>
+          <t>_res_</t>
+        </is>
+      </c>
+    </row>
+    <row r="118">
+      <c r="H118" s="4" t="inlineStr">
+        <is>
+          <t>Codes</t>
+        </is>
+      </c>
+      <c r="I118" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="119">
+      <c r="B119" s="1" t="inlineStr">
+        <is>
+          <t>Rules String selectByDate(Date[] dates)</t>
+        </is>
+      </c>
+      <c r="C119" s="2" t="n"/>
+      <c r="H119" s="5" t="inlineStr">
+        <is>
+          <t>GDHIS</t>
+        </is>
+      </c>
+      <c r="I119" s="5" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+    </row>
+    <row r="120">
+      <c r="B120" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C120" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+      <c r="H120" s="5" t="inlineStr">
+        <is>
+          <t>GADS,GDHIS</t>
+        </is>
+      </c>
+      <c r="I120" s="5" t="inlineStr">
+        <is>
+          <t>Accident</t>
+        </is>
+      </c>
+    </row>
+    <row r="121">
+      <c r="B121" s="4" t="inlineStr">
+        <is>
+          <t>contains(dates, date)</t>
+        </is>
+      </c>
+      <c r="C121" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+      <c r="H121" s="6" t="n"/>
+      <c r="I121" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="122">
+      <c r="B122" s="4" t="inlineStr">
+        <is>
+          <t>Date date</t>
+        </is>
+      </c>
+      <c r="C122" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="123">
+      <c r="B123" s="4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+      <c r="C123" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="124">
+      <c r="B124" s="5" t="inlineStr">
+        <is>
+          <t>01/02/2020</t>
+        </is>
+      </c>
+      <c r="C124" s="5" t="inlineStr">
+        <is>
+          <t>First</t>
+        </is>
+      </c>
+    </row>
+    <row r="125">
+      <c r="B125" s="5" t="inlineStr">
+        <is>
+          <t>03/04/2020</t>
+        </is>
+      </c>
+      <c r="C125" s="5" t="inlineStr">
+        <is>
+          <t>Second</t>
+        </is>
+      </c>
+    </row>
+    <row r="126">
+      <c r="B126" s="6" t="n"/>
+      <c r="C126" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
+    <row r="127"/>
+    <row r="128"/>
+    <row r="129"/>
+    <row r="130">
+      <c r="B130" s="1" t="inlineStr">
+        <is>
+          <t>Datatype CoverageCode &lt;String&gt;</t>
+        </is>
+      </c>
+      <c r="C130" s="2" t="n"/>
+    </row>
+    <row r="131">
+      <c r="B131" s="5" t="inlineStr">
+        <is>
+          <t>GADS</t>
+        </is>
+      </c>
+    </row>
+    <row r="132">
+      <c r="B132" s="5" t="inlineStr">
+        <is>
+          <t>GDHIS</t>
+        </is>
+      </c>
+    </row>
+    <row r="133"/>
+    <row r="134"/>
+    <row r="135"/>
+    <row r="136">
+      <c r="B136" s="1" t="inlineStr">
+        <is>
+          <t>Rules String selectByCoverageCode(String[] codes)</t>
+        </is>
+      </c>
+      <c r="C136" s="2" t="n"/>
+    </row>
+    <row r="137">
+      <c r="B137" s="3" t="inlineStr">
+        <is>
+          <t>C1</t>
+        </is>
+      </c>
+      <c r="C137" s="3" t="inlineStr">
+        <is>
+          <t>RET1</t>
+        </is>
+      </c>
+    </row>
+    <row r="138">
+      <c r="B138" s="4" t="inlineStr">
+        <is>
+          <t>contains(codes, code)</t>
+        </is>
+      </c>
+      <c r="C138" s="4" t="inlineStr">
+        <is>
+          <t>res</t>
+        </is>
+      </c>
+    </row>
+    <row r="139">
+      <c r="B139" s="4" t="inlineStr">
+        <is>
+          <t>CoverageCode code</t>
+        </is>
+      </c>
+      <c r="C139" s="4" t="inlineStr">
+        <is>
+          <t>String res</t>
+        </is>
+      </c>
+    </row>
+    <row r="140">
+      <c r="B140" s="4" t="inlineStr">
+        <is>
+          <t>Code</t>
+        </is>
+      </c>
+      <c r="C140" s="4" t="inlineStr">
+        <is>
+          <t>Result</t>
+        </is>
+      </c>
+    </row>
+    <row r="141">
+      <c r="B141" s="5" t="inlineStr">
+        <is>
+          <t>GADS</t>
+        </is>
+      </c>
+      <c r="C141" s="5" t="inlineStr">
+        <is>
+          <t>Accident</t>
+        </is>
+      </c>
+    </row>
+    <row r="142">
+      <c r="B142" s="5" t="inlineStr">
+        <is>
+          <t>GDHIS</t>
+        </is>
+      </c>
+      <c r="C142" s="5" t="inlineStr">
+        <is>
+          <t>Health</t>
+        </is>
+      </c>
+    </row>
+    <row r="143">
+      <c r="B143" s="6" t="n"/>
+      <c r="C143" s="5" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <mergeCells count="13">
-    <mergeCell ref="B13:C13"/>
-    <mergeCell ref="H38:J38"/>
+  <mergeCells count="25">
+    <mergeCell ref="B97:C97"/>
+    <mergeCell ref="B81:C81"/>
     <mergeCell ref="B2:C2"/>
-    <mergeCell ref="H2:I2"/>
     <mergeCell ref="B37:D37"/>
     <mergeCell ref="H59:I59"/>
-    <mergeCell ref="H16:I16"/>
+    <mergeCell ref="B86:C86"/>
+    <mergeCell ref="B130:C130"/>
+    <mergeCell ref="B136:C136"/>
+    <mergeCell ref="H98:I98"/>
     <mergeCell ref="H49:I49"/>
     <mergeCell ref="B60:C60"/>
+    <mergeCell ref="H89:I89"/>
+    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="B119:C119"/>
+    <mergeCell ref="B13:C13"/>
+    <mergeCell ref="H2:I2"/>
+    <mergeCell ref="H16:I16"/>
     <mergeCell ref="H73"/>
+    <mergeCell ref="B108:C108"/>
     <mergeCell ref="H26:J26"/>
+    <mergeCell ref="H80:I80"/>
     <mergeCell ref="B49:C49"/>
-    <mergeCell ref="B24:D24"/>
+    <mergeCell ref="H38:J38"/>
+    <mergeCell ref="H116:I116"/>
+    <mergeCell ref="H107:I107"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>